<commit_message>
Add GBS waterfall chart and Mekko chart
- Chart 1 redesigned as proper GBS scope waterfall: floating gray bars
  show scope reductions (Process standardization -21, Strategic importance -21,
  System limitations -22) with stacked colored milestone columns
  using exact data from original McKinsey chart (193→129→95→34 FTE)
- Chart 6 (new): Mekko/Marimekko chart – Market Landscape by Region & Product Line
  Excel: 100% stacked column with market size annotations
  PowerPoint: true variable-width Mekko drawn with proportional rectangles

https://claude.ai/code/session_01Di57Cqdfup39DVN9Mc9hXr
</commit_message>
<xml_diff>
--- a/McKinsey_Charts.xlsx
+++ b/McKinsey_Charts.xlsx
@@ -7,59 +7,76 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="1 Stacked Bar" sheetId="1" r:id="rId1"/>
+    <sheet name="1 GBS Waterfall" sheetId="1" r:id="rId1"/>
     <sheet name="2 Diverging Bar" sheetId="2" r:id="rId2"/>
     <sheet name="3 Scatter Line" sheetId="3" r:id="rId3"/>
     <sheet name="4 Doughnut" sheetId="4" r:id="rId4"/>
     <sheet name="5 Range Column" sheetId="5" r:id="rId5"/>
+    <sheet name="6 Mekko" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="95">
   <si>
     <t>Global Business Services Scope</t>
   </si>
   <si>
-    <t>~FTE involved in scope definition process</t>
-  </si>
-  <si>
-    <t>Stage</t>
+    <t>FTE</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Spacer</t>
+  </si>
+  <si>
+    <t>Reduction</t>
+  </si>
+  <si>
+    <t>Accounting</t>
+  </si>
+  <si>
+    <t>Customer Service</t>
+  </si>
+  <si>
+    <t>Procurement</t>
   </si>
   <si>
     <t>Sales Support</t>
   </si>
   <si>
-    <t>Procurement</t>
-  </si>
-  <si>
-    <t>Customer Service</t>
-  </si>
-  <si>
-    <t>Accounting</t>
-  </si>
-  <si>
-    <t>Benchmark scope</t>
-  </si>
-  <si>
-    <t>Process standardization</t>
-  </si>
-  <si>
-    <t>Strategic importance</t>
-  </si>
-  <si>
-    <t>System limitations</t>
-  </si>
-  <si>
-    <t>Signed-off scope</t>
-  </si>
-  <si>
-    <t>Transferred to date</t>
-  </si>
-  <si>
-    <t>To be transferred</t>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Benchmark
+scope</t>
+  </si>
+  <si>
+    <t>Process
+standardization</t>
+  </si>
+  <si>
+    <t>Strategic
+importance</t>
+  </si>
+  <si>
+    <t>System
+limitations</t>
+  </si>
+  <si>
+    <t>Signed-off
+scope</t>
+  </si>
+  <si>
+    <t>Transferred
+to date</t>
+  </si>
+  <si>
+    <t>To be
+transferred</t>
   </si>
   <si>
     <t>Source: Internal HR data</t>
@@ -245,6 +262,57 @@
   </si>
   <si>
     <t>Source: Logistics Operations Data 2024</t>
+  </si>
+  <si>
+    <t>Market Landscape by Region &amp; Product Line</t>
+  </si>
+  <si>
+    <t>Column width = market size ($M)  |  Height = share within region (%)</t>
+  </si>
+  <si>
+    <t>Product Line</t>
+  </si>
+  <si>
+    <t>Europe</t>
+  </si>
+  <si>
+    <t>North America</t>
+  </si>
+  <si>
+    <t>Asia Pacific</t>
+  </si>
+  <si>
+    <t>Rest of World</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>Mid-Range</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Market size ($M)</t>
+  </si>
+  <si>
+    <t>$320M</t>
+  </si>
+  <si>
+    <t>$480M</t>
+  </si>
+  <si>
+    <t>$260M</t>
+  </si>
+  <si>
+    <t>$140M</t>
+  </si>
+  <si>
+    <t>Note: Column widths equal in Excel; see PowerPoint for proportional Mekko</t>
+  </si>
+  <si>
+    <t>Source: Market Intelligence Report 2024</t>
   </si>
 </sst>
 </file>
@@ -255,7 +323,7 @@
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -330,6 +398,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF002060"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -396,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -433,6 +508,9 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,21 +528,293 @@
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="bar"/>
+        <c:barDir val="col"/>
         <c:grouping val="stacked"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
+            <c:v>Spacer</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="FFFFFF"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls/>
+          <c:cat>
             <c:strRef>
-              <c:f>'1 Stacked Bar'!$C$5</c:f>
+              <c:f>'1 GBS Waterfall'!$B$6:$B$12</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Sales Support</c:v>
+                  <c:v>Benchmark
+scope</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Process
+standardization</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Strategic
+importance</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>System
+limitations</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Signed-off
+scope</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Transferred
+to date</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>To be
+transferred</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'1 GBS Waterfall'!$C$6:$C$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>172</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>151</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Scope reduction</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="D9D9D9"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="7F7F7F"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'1 GBS Waterfall'!$B$6:$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>Benchmark
+scope</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Process
+standardization</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Strategic
+importance</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>System
+limitations</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Signed-off
+scope</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Transferred
+to date</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>To be
+transferred</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'1 GBS Waterfall'!$D$6:$D$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Accounting</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'1 GBS Waterfall'!$B$6:$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>Benchmark
+scope</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Process
+standardization</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Strategic
+importance</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>System
+limitations</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Signed-off
+scope</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Transferred
+to date</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>To be
+transferred</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'1 GBS Waterfall'!$E$6:$E$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>66</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Customer Service</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -480,7 +830,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="800" baseline="0">
+                  <a:defRPr sz="900" b="1" baseline="0">
                     <a:solidFill>
                       <a:srgbClr val="FFFFFF"/>
                     </a:solidFill>
@@ -494,77 +844,76 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'1 Stacked Bar'!$B$6:$B$12</c:f>
+              <c:f>'1 GBS Waterfall'!$B$6:$B$12</c:f>
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Benchmark scope</c:v>
+                  <c:v>Benchmark
+scope</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Process standardization</c:v>
+                  <c:v>Process
+standardization</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Strategic importance</c:v>
+                  <c:v>Strategic
+importance</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>System limitations</c:v>
+                  <c:v>System
+limitations</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Signed-off scope</c:v>
+                  <c:v>Signed-off
+scope</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Transferred to date</c:v>
+                  <c:v>Transferred
+to date</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>To be transferred</c:v>
+                  <c:v>To be
+transferred</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'1 Stacked Bar'!$C$6:$C$12</c:f>
+              <c:f>'1 GBS Waterfall'!$F$6:$F$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>450</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>380</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>320</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>280</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>250</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>180</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>120</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
         <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
+          <c:idx val="4"/>
+          <c:order val="4"/>
           <c:tx>
-            <c:strRef>
-              <c:f>'1 Stacked Bar'!$D$5</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Procurement</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>Procurement</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -580,7 +929,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="800" baseline="0">
+                  <a:defRPr sz="900" b="1" baseline="0">
                     <a:solidFill>
                       <a:srgbClr val="FFFFFF"/>
                     </a:solidFill>
@@ -594,77 +943,76 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'1 Stacked Bar'!$B$6:$B$12</c:f>
+              <c:f>'1 GBS Waterfall'!$B$6:$B$12</c:f>
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Benchmark scope</c:v>
+                  <c:v>Benchmark
+scope</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Process standardization</c:v>
+                  <c:v>Process
+standardization</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Strategic importance</c:v>
+                  <c:v>Strategic
+importance</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>System limitations</c:v>
+                  <c:v>System
+limitations</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Signed-off scope</c:v>
+                  <c:v>Signed-off
+scope</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Transferred to date</c:v>
+                  <c:v>Transferred
+to date</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>To be transferred</c:v>
+                  <c:v>To be
+transferred</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'1 Stacked Bar'!$D$6:$D$12</c:f>
+              <c:f>'1 GBS Waterfall'!$G$6:$G$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>120</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>90</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>80</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>70</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>45</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>30</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:idx val="5"/>
+          <c:order val="5"/>
           <c:tx>
-            <c:strRef>
-              <c:f>'1 Stacked Bar'!$E$5</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Customer Service</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>Sales Support</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -680,7 +1028,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="800" baseline="0">
+                  <a:defRPr sz="900" b="1" baseline="0">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -694,159 +1042,66 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'1 Stacked Bar'!$B$6:$B$12</c:f>
+              <c:f>'1 GBS Waterfall'!$B$6:$B$12</c:f>
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Benchmark scope</c:v>
+                  <c:v>Benchmark
+scope</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Process standardization</c:v>
+                  <c:v>Process
+standardization</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Strategic importance</c:v>
+                  <c:v>Strategic
+importance</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>System limitations</c:v>
+                  <c:v>System
+limitations</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Signed-off scope</c:v>
+                  <c:v>Signed-off
+scope</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Transferred to date</c:v>
+                  <c:v>Transferred
+to date</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>To be transferred</c:v>
+                  <c:v>To be
+transferred</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'1 Stacked Bar'!$E$6:$E$12</c:f>
+              <c:f>'1 GBS Waterfall'!$H$6:$H$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>180</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>150</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>130</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>110</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>100</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>70</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>45</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'1 Stacked Bar'!$F$5</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Accounting</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="D9D9D9"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:dLbls>
-            <c:txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="800" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:showVal val="1"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'1 Stacked Bar'!$B$6:$B$12</c:f>
-              <c:strCache>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>Benchmark scope</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Process standardization</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Strategic importance</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>System limitations</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Signed-off scope</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Transferred to date</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>To be transferred</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'1 Stacked Bar'!$F$6:$F$12</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>200</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>170</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>130</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>90</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>60</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -859,13 +1114,15 @@
       <c:catAx>
         <c:axId val="50010001"/>
         <c:scaling>
-          <c:orientation val="maxMin"/>
+          <c:orientation val="minMax"/>
         </c:scaling>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:ln>
-            <a:noFill/>
+            <a:solidFill>
+              <a:srgbClr val="7F7F7F"/>
+            </a:solidFill>
           </a:ln>
         </c:spPr>
         <c:txPr>
@@ -873,7 +1130,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="800" baseline="0">
+              <a:defRPr sz="900" b="1" baseline="0">
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
@@ -890,8 +1147,10 @@
         <c:axId val="50010002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="220"/>
+          <c:min val="0"/>
         </c:scaling>
-        <c:axPos val="t"/>
+        <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="6350">
@@ -935,6 +1194,10 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="0"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
       <c:layout/>
       <c:txPr>
         <a:bodyPr/>
@@ -3018,19 +3281,472 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="percentStacked"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'6 Mekko'!$B$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Premium</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showPercent val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'6 Mekko'!$C$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Europe</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>North America</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Asia Pacific</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Rest of World</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'6 Mekko'!$C$6:$F$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.35</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'6 Mekko'!$B$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Mid-Range</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F5FA6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showPercent val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'6 Mekko'!$C$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Europe</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>North America</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Asia Pacific</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Rest of World</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'6 Mekko'!$C$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.35</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'6 Mekko'!$B$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Value</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="9DC3E6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showPercent val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'6 Mekko'!$C$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Europe</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>North America</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Asia Pacific</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Rest of World</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'6 Mekko'!$C$8:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.35</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'6 Mekko'!$B$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Other</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="D9D9D9"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showPercent val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'6 Mekko'!$C$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Europe</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>North America</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Asia Pacific</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Rest of World</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'6 Mekko'!$C$9:$F$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.15</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:overlap val="100"/>
+        <c:axId val="50080001"/>
+        <c:axId val="50080002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50080001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="1" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50080002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50080002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50080001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" baseline="0">
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3231,6 +3947,41 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>428625</xdr:colOff>
       <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3538,15 +4289,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B2:G31"/>
+  <dimension ref="B2:I35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="0.85546875" customWidth="1"/>
-    <col min="2" max="2" width="26.7109375" customWidth="1"/>
-    <col min="3" max="7" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="9" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7">
+    <row r="2" spans="2:9">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3555,13 +4306,15 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="2:7">
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="2:9">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:9">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -3577,134 +4330,206 @@
       <c r="F5" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="2:7">
+      <c r="G5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9">
       <c r="B6" s="4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6" s="5">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="D6" s="5">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="E6" s="5">
-        <v>180</v>
+        <v>89</v>
       </c>
       <c r="F6" s="5">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7">
+        <v>45</v>
+      </c>
+      <c r="G6" s="5">
+        <v>34</v>
+      </c>
+      <c r="H6" s="5">
+        <v>25</v>
+      </c>
+      <c r="I6" s="5">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9">
       <c r="B7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="5">
+        <v>172</v>
+      </c>
+      <c r="D7" s="5">
+        <v>21</v>
+      </c>
+      <c r="E7" s="5">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9">
+      <c r="B8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="5">
+        <v>151</v>
+      </c>
+      <c r="D8" s="5">
+        <v>21</v>
+      </c>
+      <c r="E8" s="5">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9">
+      <c r="B9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5">
+        <v>129</v>
+      </c>
+      <c r="D9" s="5">
+        <v>22</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9">
+      <c r="B10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>66</v>
+      </c>
+      <c r="F10" s="5">
+        <v>31</v>
+      </c>
+      <c r="G10" s="5">
+        <v>19</v>
+      </c>
+      <c r="H10" s="5">
+        <v>13</v>
+      </c>
+      <c r="I10" s="5">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9">
+      <c r="B11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>45</v>
+      </c>
+      <c r="F11" s="5">
+        <v>23</v>
+      </c>
+      <c r="G11" s="5">
+        <v>19</v>
+      </c>
+      <c r="H11" s="5">
         <v>8</v>
       </c>
-      <c r="C7" s="5">
-        <v>380</v>
-      </c>
-      <c r="D7" s="5">
-        <v>90</v>
-      </c>
-      <c r="E7" s="5">
-        <v>150</v>
-      </c>
-      <c r="F7" s="5">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7">
-      <c r="B8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="5">
-        <v>320</v>
-      </c>
-      <c r="D8" s="5">
-        <v>80</v>
-      </c>
-      <c r="E8" s="5">
-        <v>130</v>
-      </c>
-      <c r="F8" s="5">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7">
-      <c r="B9" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="5">
-        <v>280</v>
-      </c>
-      <c r="D9" s="5">
-        <v>70</v>
-      </c>
-      <c r="E9" s="5">
-        <v>110</v>
-      </c>
-      <c r="F9" s="5">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7">
-      <c r="B10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="5">
-        <v>250</v>
-      </c>
-      <c r="D10" s="5">
-        <v>60</v>
-      </c>
-      <c r="E10" s="5">
-        <v>100</v>
-      </c>
-      <c r="F10" s="5">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7">
-      <c r="B11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="5">
-        <v>180</v>
-      </c>
-      <c r="D11" s="5">
-        <v>45</v>
-      </c>
-      <c r="E11" s="5">
-        <v>70</v>
-      </c>
-      <c r="F11" s="5">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7">
+      <c r="I11" s="5">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9">
       <c r="B12" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C12" s="5">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="D12" s="5">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E12" s="5">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="F12" s="5">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="31" spans="2:2">
-      <c r="B31" s="6" t="s">
-        <v>14</v>
+        <v>8</v>
+      </c>
+      <c r="G12" s="5">
+        <v>5</v>
+      </c>
+      <c r="H12" s="5">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3723,7 +4548,7 @@
   <sheetData>
     <row r="2" spans="2:8">
       <c r="B2" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3734,32 +4559,32 @@
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="2:8">
       <c r="B5" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="2:8">
       <c r="B6" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C6" s="7">
         <v>-0.15</v>
@@ -3774,12 +4599,12 @@
         <v>0.25</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="2:8">
       <c r="B7" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C7" s="7">
         <v>-0.1</v>
@@ -3794,12 +4619,12 @@
         <v>0.3</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="2:8">
       <c r="B8" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C8" s="7">
         <v>-0.22</v>
@@ -3814,12 +4639,12 @@
         <v>0.25</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="2:8">
       <c r="B9" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C9" s="7">
         <v>-0.05</v>
@@ -3834,12 +4659,12 @@
         <v>0.33</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="2:8">
       <c r="B10" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C10" s="7">
         <v>-0.26</v>
@@ -3854,12 +4679,12 @@
         <v>0.27</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="2:8">
       <c r="B11" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C11" s="7">
         <v>-0.12</v>
@@ -3874,12 +4699,12 @@
         <v>0.33</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="2:2">
       <c r="B27" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -3902,7 +4727,7 @@
   <sheetData>
     <row r="2" spans="2:9">
       <c r="B2" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3914,27 +4739,27 @@
     </row>
     <row r="3" spans="2:9">
       <c r="B3" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="2:9">
       <c r="B5" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="2:9">
@@ -4049,7 +4874,7 @@
     </row>
     <row r="28" spans="2:2">
       <c r="B28" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -4072,7 +4897,7 @@
   <sheetData>
     <row r="2" spans="2:13">
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4088,38 +4913,38 @@
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="2:13">
       <c r="B5" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K5" s="3"/>
     </row>
     <row r="6" spans="2:13">
       <c r="B6" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C6" s="7">
         <v>0.35</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G6" s="7">
         <v>0.38</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="K6" s="7">
         <v>0.42</v>
@@ -4127,19 +4952,19 @@
     </row>
     <row r="7" spans="2:13">
       <c r="B7" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C7" s="7">
         <v>0.2</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G7" s="7">
         <v>0.22</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K7" s="7">
         <v>0.19</v>
@@ -4147,19 +4972,19 @@
     </row>
     <row r="8" spans="2:13">
       <c r="B8" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C8" s="7">
         <v>0.18</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G8" s="7">
         <v>0.16</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="K8" s="7">
         <v>0.15</v>
@@ -4167,19 +4992,19 @@
     </row>
     <row r="9" spans="2:13">
       <c r="B9" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C9" s="7">
         <v>0.12</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G9" s="7">
         <v>0.11</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="K9" s="7">
         <v>0.1</v>
@@ -4187,19 +5012,19 @@
     </row>
     <row r="10" spans="2:13">
       <c r="B10" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C10" s="7">
         <v>0.09</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G10" s="7">
         <v>0.08</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K10" s="7">
         <v>0.09</v>
@@ -4207,19 +5032,19 @@
     </row>
     <row r="11" spans="2:13">
       <c r="B11" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C11" s="7">
         <v>0.06</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G11" s="7">
         <v>0.05</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="K11" s="7">
         <v>0.05</v>
@@ -4227,32 +5052,32 @@
     </row>
     <row r="28" spans="2:7">
       <c r="B28" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="2:7">
       <c r="B29" s="10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="2:7">
       <c r="B31" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -4278,7 +5103,7 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4291,32 +5116,32 @@
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C6" s="5">
         <v>80</v>
@@ -4336,7 +5161,7 @@
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C7" s="5">
         <v>85</v>
@@ -4356,7 +5181,7 @@
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C8" s="5">
         <v>78</v>
@@ -4376,7 +5201,7 @@
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C9" s="5">
         <v>90</v>
@@ -4396,7 +5221,7 @@
     </row>
     <row r="10" spans="2:10">
       <c r="B10" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C10" s="5">
         <v>88</v>
@@ -4416,7 +5241,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C11" s="5">
         <v>82</v>
@@ -4436,7 +5261,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="B12" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C12" s="5">
         <v>95</v>
@@ -4456,7 +5281,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="B13" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C13" s="5">
         <v>91</v>
@@ -4476,7 +5301,7 @@
     </row>
     <row r="32" spans="2:2">
       <c r="B32" s="6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -4486,4 +5311,163 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="B2:F21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="0.85546875" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="6" width="14.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6">
+      <c r="B2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="2:6">
+      <c r="B3" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6">
+      <c r="C4" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6">
+      <c r="B5" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6">
+      <c r="B6" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="D6" s="7">
+        <v>0.35</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="F6" s="7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6">
+      <c r="B7" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="D7" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="E7" s="7">
+        <v>0.35</v>
+      </c>
+      <c r="F7" s="7">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6">
+      <c r="B8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="F8" s="7">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6">
+      <c r="B9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="D9" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="E9" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="7">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6">
+      <c r="B11" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="5">
+        <v>320</v>
+      </c>
+      <c r="D11" s="5">
+        <v>480</v>
+      </c>
+      <c r="E11" s="5">
+        <v>260</v>
+      </c>
+      <c r="F11" s="5">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 6 new chart types (charts 7-12) to Excel and PowerPoint outputs
Adds the following new charts to both McKinsey_Charts.xlsx and McKinsey_Slides.pptx:
- Chart 7: 2x2 Priority Matrix (scatter plot with quadrant backgrounds)
- Chart 8: EBITDA Bridge (horizontal waterfall with up/down color coding)
- Chart 9: Gantt / Transformation Roadmap (stacked bar Gantt chart)
- Chart 10: Harvey Balls capability benchmarking matrix
- Chart 11: Tornado / Sensitivity Analysis (diverging bar chart)
- Chart 12: Income Statement Sankey (matplotlib PNG, gracefully skipped if not installed)

Also adds _make_sankey_png() as a module-level function and updates the
docstring to reflect 12 charts. Uses correct python-pptx FreeformBuilder
API (add_line_segments) for Harvey Ball partial fills.

https://claude.ai/code/session_01Di57Cqdfup39DVN9Mc9hXr
</commit_message>
<xml_diff>
--- a/McKinsey_Charts.xlsx
+++ b/McKinsey_Charts.xlsx
@@ -13,13 +13,19 @@
     <sheet name="4 Doughnut" sheetId="4" r:id="rId4"/>
     <sheet name="5 Range Column" sheetId="5" r:id="rId5"/>
     <sheet name="6 Mekko" sheetId="6" r:id="rId6"/>
+    <sheet name="7_Priority_Matrix" sheetId="7" r:id="rId7"/>
+    <sheet name="8_EBITDA_Bridge" sheetId="8" r:id="rId8"/>
+    <sheet name="9_Gantt_Roadmap" sheetId="9" r:id="rId9"/>
+    <sheet name="10_Harvey_Balls" sheetId="10" r:id="rId10"/>
+    <sheet name="11_Tornado" sheetId="11" r:id="rId11"/>
+    <sheet name="12_Sankey" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="184">
   <si>
     <t>Global Business Services Scope</t>
   </si>
@@ -313,6 +319,273 @@
   </si>
   <si>
     <t>Source: Market Intelligence Report 2024</t>
+  </si>
+  <si>
+    <t>2×2 Priority Matrix</t>
+  </si>
+  <si>
+    <t>Initiative</t>
+  </si>
+  <si>
+    <t>Impl. Ease (0-10)</t>
+  </si>
+  <si>
+    <t>Business Impact (0-10)</t>
+  </si>
+  <si>
+    <t>Digital Core Platform</t>
+  </si>
+  <si>
+    <t>Customer 360</t>
+  </si>
+  <si>
+    <t>Cost Transformation</t>
+  </si>
+  <si>
+    <t>Talent Upskilling</t>
+  </si>
+  <si>
+    <t>Process Automation</t>
+  </si>
+  <si>
+    <t>Org Redesign</t>
+  </si>
+  <si>
+    <t>Analytics &amp; AI</t>
+  </si>
+  <si>
+    <t>Supplier Consolidation</t>
+  </si>
+  <si>
+    <t>ESG Reporting</t>
+  </si>
+  <si>
+    <t>Legacy Migration</t>
+  </si>
+  <si>
+    <t>Source: Strategic Planning Workshop 2024</t>
+  </si>
+  <si>
+    <t>EBITDA Bridge</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Value ($M)</t>
+  </si>
+  <si>
+    <t>Bar</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Cost of Goods Sold</t>
+  </si>
+  <si>
+    <t>Gross Profit</t>
+  </si>
+  <si>
+    <t>SG&amp;A</t>
+  </si>
+  <si>
+    <t>R&amp;D</t>
+  </si>
+  <si>
+    <t>D&amp;A Add-back</t>
+  </si>
+  <si>
+    <t>One-off Items</t>
+  </si>
+  <si>
+    <t>EBITDA</t>
+  </si>
+  <si>
+    <t>Source: Management Accounts FY2024</t>
+  </si>
+  <si>
+    <t>Transformation Roadmap</t>
+  </si>
+  <si>
+    <t>Workstream</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Start (week)</t>
+  </si>
+  <si>
+    <t>Duration (weeks)</t>
+  </si>
+  <si>
+    <t>Assessment</t>
+  </si>
+  <si>
+    <t>Current State Analysis</t>
+  </si>
+  <si>
+    <t>Stakeholder Interviews</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Future State Blueprint</t>
+  </si>
+  <si>
+    <t>Business Case</t>
+  </si>
+  <si>
+    <t>Pilot</t>
+  </si>
+  <si>
+    <t>Site Preparation</t>
+  </si>
+  <si>
+    <t>Pilot Execution</t>
+  </si>
+  <si>
+    <t>Rollout</t>
+  </si>
+  <si>
+    <t>Wave 1 Deployment</t>
+  </si>
+  <si>
+    <t>Wave 2 Deployment</t>
+  </si>
+  <si>
+    <t>Change Management</t>
+  </si>
+  <si>
+    <t>Governance</t>
+  </si>
+  <si>
+    <t>PMO &amp; Tracking</t>
+  </si>
+  <si>
+    <t>Source: Programme Management Office</t>
+  </si>
+  <si>
+    <t>Capability Benchmarking</t>
+  </si>
+  <si>
+    <t>Capability</t>
+  </si>
+  <si>
+    <t>McKinsey</t>
+  </si>
+  <si>
+    <t>BCG</t>
+  </si>
+  <si>
+    <t>Bain</t>
+  </si>
+  <si>
+    <t>Deloitte</t>
+  </si>
+  <si>
+    <t>Accenture</t>
+  </si>
+  <si>
+    <t>Strategy &amp; Vision</t>
+  </si>
+  <si>
+    <t>●</t>
+  </si>
+  <si>
+    <t>◕</t>
+  </si>
+  <si>
+    <t>Digital Capability</t>
+  </si>
+  <si>
+    <t>◑</t>
+  </si>
+  <si>
+    <t>Operational Excellence</t>
+  </si>
+  <si>
+    <t>M&amp;A Advisory</t>
+  </si>
+  <si>
+    <t>Talent &amp; Culture</t>
+  </si>
+  <si>
+    <t>Technology Delivery</t>
+  </si>
+  <si>
+    <t>Sector Expertise</t>
+  </si>
+  <si>
+    <t>Legend:</t>
+  </si>
+  <si>
+    <t>○ No capability</t>
+  </si>
+  <si>
+    <t>◔ Basic</t>
+  </si>
+  <si>
+    <t>◑ Moderate</t>
+  </si>
+  <si>
+    <t>◕ Strong</t>
+  </si>
+  <si>
+    <t>● Leading</t>
+  </si>
+  <si>
+    <t>Source: Internal capability assessment</t>
+  </si>
+  <si>
+    <t>Sensitivity Analysis – NPV Impact ($M)</t>
+  </si>
+  <si>
+    <t>Driver</t>
+  </si>
+  <si>
+    <t>Downside ($M)</t>
+  </si>
+  <si>
+    <t>Upside ($M)</t>
+  </si>
+  <si>
+    <t>Revenue growth rate</t>
+  </si>
+  <si>
+    <t>EBITDA margin</t>
+  </si>
+  <si>
+    <t>Exit multiple (EV/EBITDA)</t>
+  </si>
+  <si>
+    <t>WACC / Discount rate</t>
+  </si>
+  <si>
+    <t>Working capital intensity</t>
+  </si>
+  <si>
+    <t>Cost of goods sold</t>
+  </si>
+  <si>
+    <t>Capex intensity</t>
+  </si>
+  <si>
+    <t>Tax rate</t>
+  </si>
+  <si>
+    <t>Source: Financial model – sensitivity run</t>
+  </si>
+  <si>
+    <t>Income Statement Sankey</t>
+  </si>
+  <si>
+    <t>[Install matplotlib to see Sankey: pip install matplotlib]</t>
+  </si>
+  <si>
+    <t>Source: Company financials FY2024</t>
   </si>
 </sst>
 </file>
@@ -323,7 +596,7 @@
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -405,6 +678,32 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF002060"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF002060"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -450,7 +749,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -467,11 +766,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -509,6 +838,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1198,6 +1539,964 @@
         <c:idx val="0"/>
         <c:delete val="1"/>
       </c:legendEntry>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" baseline="0">
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>EBITDA Bridge  ($M)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Spacer</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'8_EBITDA_Bridge'!$A$3:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cost of Goods Sold</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Gross Profit</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>SG&amp;A</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>R&amp;D</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>D&amp;A Add-back</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>One-off Items</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>EBITDA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'8_EBITDA_Bridge'!$C$3:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>205</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>205</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>217</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Value</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'8_EBITDA_Bridge'!$A$3:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cost of Goods Sold</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Gross Profit</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>SG&amp;A</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>R&amp;D</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>D&amp;A Add-back</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>One-off Items</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>EBITDA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'8_EBITDA_Bridge'!$D$3:$D$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>217</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:overlap val="100"/>
+        <c:axId val="50100001"/>
+        <c:axId val="50100002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50100001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50100002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50100002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50100001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Transformation Roadmap  (weeks)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Start</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'9_Gantt_Roadmap'!$B$3:$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Current State Analysis</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Stakeholder Interviews</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Future State Blueprint</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Business Case</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Site Preparation</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Pilot Execution</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Wave 1 Deployment</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Wave 2 Deployment</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Change Management</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>PMO &amp; Tracking</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'9_Gantt_Roadmap'!$C$3:$C$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Duration</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'9_Gantt_Roadmap'!$B$3:$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Current State Analysis</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Stakeholder Interviews</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Future State Blueprint</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Business Case</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Site Preparation</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Pilot Execution</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Wave 1 Deployment</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Wave 2 Deployment</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Change Management</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>PMO &amp; Tracking</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'9_Gantt_Roadmap'!$D$3:$D$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>32</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:overlap val="100"/>
+        <c:axId val="50110001"/>
+        <c:axId val="50110002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50110001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50110002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50110002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="34"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Week</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50110001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>NPV Sensitivity  ($M)  –  Base Case = $217M</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Downside</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="800" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'11_Tornado'!$A$3:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Revenue growth rate</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>EBITDA margin</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Exit multiple (EV/EBITDA)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>WACC / Discount rate</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Working capital intensity</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cost of goods sold</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Capex intensity</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Tax rate</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'11_Tornado'!$B$3:$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>-48</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-35</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-32</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-38</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-22</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-20</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-18</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Upside</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="70AD47"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="800" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'11_Tornado'!$A$3:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Revenue growth rate</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>EBITDA margin</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Exit multiple (EV/EBITDA)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>WACC / Discount rate</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Working capital intensity</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cost of goods sold</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Capex intensity</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Tax rate</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'11_Tornado'!$C$3:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50120001"/>
+        <c:axId val="50120002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50120001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50120002"/>
+        <c:crossesAt val="0"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50120002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50120001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
       <c:layout/>
       <c:txPr>
         <a:bodyPr/>
@@ -3734,6 +5033,307 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>2×2 Initiative Priority Matrix</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Initiatives</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="002060"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'7_Priority_Matrix'!$B$3:$B$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'7_Priority_Matrix'!$C$3:$C$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>9.5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>_ref_v</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="12700">
+              <a:solidFill>
+                <a:srgbClr val="7F7F7F"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'7_Priority_Matrix'!$B$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'7_Priority_Matrix'!$B$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:axId val="50090001"/>
+        <c:axId val="50090002"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="50090001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="10"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" baseline="0">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+                    <a:latin typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Implementation Ease →</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50090002"/>
+        <c:crossesAt val="5"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="50090002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="10"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" baseline="0">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+                    <a:latin typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Business Impact →</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50090001"/>
+        <c:crossesAt val="5"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="D9D9D9"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -3747,6 +5347,41 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>438150</xdr:colOff>
       <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3982,6 +5617,111 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>314325</xdr:colOff>
       <xdr:row>33</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4536,6 +6276,368 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF9DC3E6"/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="6" width="14.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="22" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="26" customHeight="1">
+      <c r="A3" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="26" customHeight="1">
+      <c r="A4" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="26" customHeight="1">
+      <c r="A5" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="26" customHeight="1">
+      <c r="A6" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="26" customHeight="1">
+      <c r="A7" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="26" customHeight="1">
+      <c r="A8" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="26" customHeight="1">
+      <c r="A9" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF002060"/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3" s="5">
+        <v>-48</v>
+      </c>
+      <c r="C3" s="5">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4" s="5">
+        <v>-35</v>
+      </c>
+      <c r="C4" s="5">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" s="5">
+        <v>-32</v>
+      </c>
+      <c r="C5" s="5">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" s="5">
+        <v>-38</v>
+      </c>
+      <c r="C6" s="5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="5">
+        <v>-22</v>
+      </c>
+      <c r="C7" s="5">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" s="5">
+        <v>-20</v>
+      </c>
+      <c r="C8" s="5">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="5">
+        <v>-18</v>
+      </c>
+      <c r="C9" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B10" s="5">
+        <v>-14</v>
+      </c>
+      <c r="C10" s="5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF1F5FA6"/>
+  </sheetPr>
+  <dimension ref="A1:A61"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="6" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="6" t="s">
+        <v>183</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:H27"/>
@@ -5470,4 +7572,490 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF1F5FA6"/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="5">
+        <v>8</v>
+      </c>
+      <c r="C3" s="5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="5">
+        <v>6.5</v>
+      </c>
+      <c r="C4" s="5">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="C5" s="5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="C6" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="5">
+        <v>8.5</v>
+      </c>
+      <c r="C7" s="5">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="5">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="5">
+        <v>5.5</v>
+      </c>
+      <c r="C9" s="5">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" s="5">
+        <v>7</v>
+      </c>
+      <c r="C10" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="5">
+        <v>6</v>
+      </c>
+      <c r="C11" s="5">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="C12" s="5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF002060"/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="4" width="10.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="5">
+        <v>500</v>
+      </c>
+      <c r="C3" s="5">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="5">
+        <v>-180</v>
+      </c>
+      <c r="C4" s="5">
+        <v>320</v>
+      </c>
+      <c r="D4" s="5">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B5" s="5">
+        <v>320</v>
+      </c>
+      <c r="C5" s="5">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="5">
+        <v>-70</v>
+      </c>
+      <c r="C6" s="5">
+        <v>250</v>
+      </c>
+      <c r="D6" s="5">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="5">
+        <v>-45</v>
+      </c>
+      <c r="C7" s="5">
+        <v>205</v>
+      </c>
+      <c r="D7" s="5">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="5">
+        <v>32</v>
+      </c>
+      <c r="C8" s="5">
+        <v>205</v>
+      </c>
+      <c r="D8" s="5">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="5">
+        <v>-20</v>
+      </c>
+      <c r="C9" s="5">
+        <v>217</v>
+      </c>
+      <c r="D9" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" s="5">
+        <v>217</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF1F5FA6"/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" customWidth="1"/>
+    <col min="3" max="4" width="10.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="5">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2</v>
+      </c>
+      <c r="D4" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="5">
+        <v>5</v>
+      </c>
+      <c r="D5" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="5">
+        <v>7</v>
+      </c>
+      <c r="D6" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C7" s="5">
+        <v>12</v>
+      </c>
+      <c r="D7" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8" s="5">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C9" s="5">
+        <v>19</v>
+      </c>
+      <c r="D9" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" s="5">
+        <v>25</v>
+      </c>
+      <c r="D10" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="5">
+        <v>19</v>
+      </c>
+      <c r="D11" s="5">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>